<commit_message>
docs(planning): record FOUND-002 completion and correct FOUND-001 status
Fills the FOUND-002 row in DEVELOPMENT_PROGRESS.xlsx, adds CHG-001
(FOUND-002 implementation) and CHG-002 (FOUND-001 status correction)
to CHANGE_LOG.xlsx, and adds a DEVELOPMENT_LOG.md entry making the
correction explicit: MASTER_TASK_LIST.xlsx's Status column for
FOUND-001 was NOT_STARTED despite the task being fully implemented
and committed on 2026-09-10 - only DEVELOPMENT_PROGRESS.xlsx was
updated at the time. Both FOUND-001 and FOUND-002 are now COMPLETED
in MASTER_TASK_LIST.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -482,8 +482,112 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHG-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FOUND-002</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Implemented Express 5 API foundation (ESM/NodeNext): standardized response envelope, request ID, pino logging, zod-validated env config, CORS/helmet, in-memory rate-limit foundation, graceful shutdown, GET /api/v1/health.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Establish the backend platform foundation required before any business module (auth, catalog, commerce, etc.) can be built, per MASTER_TASK_LIST FOUND-002.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>New apps/api runtime dependencies (Express, helmet, cors, pino, pino-http, zod, express-rate-limit); apps/api switched from CommonJS/Node16 to ESM/NodeNext; shared packages/config/eslint/base.mjs gained a no-unused-vars exception for underscore-prefixed params.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business logic, no DB/auth/RBAC. Rate limiter is single-instance only (documented, not yet wired to any route).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved across 3 rounds before execution</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>f0ff3a46bfc30b95aef0b6b0cf42d7e9adca4635</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHG-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FOUND-001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Corrected Planning/MASTER_TASK_LIST.xlsx Status column for FOUND-001 from NOT_STARTED to COMPLETED.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FOUND-001 was fully implemented, validated, and committed (commits d025c01, 7ffbc53) on 2026-09-10, but the Status column in MASTER_TASK_LIST.xlsx was never updated at completion time - only DEVELOPMENT_PROGRESS.xlsx was. Data-integrity correction, not a re-implementation.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Planning-data only; no code impact.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>None - documentation/tracking correction.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>d025c01 (original FOUND-001 implementation); correction recorded alongside the FOUND-002 planning-docs commit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record DB-001 completion
Fills the DB-001 row in DEVELOPMENT_PROGRESS.xlsx, adds CHG-003 to
CHANGE_LOG.xlsx, marks DB-001 COMPLETED in MASTER_TASK_LIST.xlsx,
records DEC-006 (migration tool choice, deliberately deferred) in
OPEN_DECISIONS.md, and adds a DEVELOPMENT_LOG.md entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -586,8 +586,60 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CHG-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DB-001</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Implemented MongoDB connection foundation: singleton Mongoose connection with bounded initial-connect retry, sanitizeFilter/strictQuery, dev-only autoIndex/autoCreate, global maxTimeMS plugin, withTransaction() helper (MongoDB-only), GET /api/v1/ready, production TLS/localhost startup safety guards.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Establish the database platform foundation required before any business schema (catalog, inventory, orders, etc.) can be built, per MASTER_TASK_LIST DB-001, extending FOUND-002 rather than redesigning it.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>New apps/api dependencies (mongoose, mongodb-memory-server); apps/api/src/config/env.ts and index.ts modified to integrate DB connect/disconnect into the existing FOUND-002 boot/shutdown sequence; new GET /api/v1/ready endpoint and NOT_READY error code.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business schemas, no auth/RBAC, no Redis. withTransaction() explicitly documented as MongoDB-only, not atomic with external side effects.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved with 2 explicit confirmations before execution</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0ce5ed8786eebcefa7e37316d2d9f0b5c419745e</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record CAT-001 completion
Fills the CAT-001 row in DEVELOPMENT_PROGRESS.xlsx, marks CAT-001
COMPLETED in MASTER_TASK_LIST.xlsx (Status only - roadmap wording for
CAT-001/002/003/004 is unchanged), adds CHG-004 to CHANGE_LOG.xlsx,
records ADR-009 through ADR-012 in ARCHITECTURE_DECISIONS.md, and adds
a DEVELOPMENT_LOG.md entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -638,8 +638,60 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CHG-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CAT-001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Implemented the Category domain foundation only: Mongoose model, repository, and service (Service -&gt; Repository -&gt; Model), organization-scoped hierarchy with cycle/cross-org prevention, soft-archive lifecycle, hand-rolled slug generation with database-enforced uniqueness. No HTTP routes/controllers, no Brand/Product/Variant.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Establish the Category foundation per MASTER_TASK_LIST CAT-001, without inventing a temporary authentication/authorization system while SEC-001/SEC-002 remain NOT_STARTED, and without broadening scope into CAT-002/003/004 territory (an earlier, broader combined-catalog proposal was explicitly rejected by the developer in favor of keeping the existing task boundaries intact).</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/catalog/ directory (10 files, all new); no existing file modified; no new dependency; no route registered in app.ts/routes.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business CRUD exposed over HTTP yet, no auth/RBAC. Routes/controllers remain deferred until SEC-002.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved across 3 rounds (initial broad proposal rejected and narrowed, then the narrowed plan approved) before execution</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>b332de98c3133920a0c0626efb18309e6a2af2f3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record CAT-002 completion
Fills the CAT-002 row in DEVELOPMENT_PROGRESS.xlsx, marks CAT-002
COMPLETED in MASTER_TASK_LIST.xlsx (Status only - roadmap wording for
CAT-001/002/003/004 is unchanged), adds CHG-005 to CHANGE_LOG.xlsx,
and adds a DEVELOPMENT_LOG.md entry. No new ADRs - ADR-009/011/012
already covered Brand.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -690,8 +690,60 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CHG-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CAT-002</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Implemented the Brand domain foundation: Mongoose model, repository, and service (Service -&gt; Repository -&gt; Model), organization-scoped slug uniqueness, soft-archive lifecycle, logo reference (no upload/storage infrastructure). Extracted the shared isDuplicateKeyError() helper from CAT-001's category.repository.ts into apps/api/src/modules/catalog/lib/mongo-errors.ts, now used by both Category and Brand repositories.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Establish the Brand foundation per MASTER_TASK_LIST CAT-002, reusing CAT-001 conventions (slugify, common validation helpers, lifecycle enum shape) without inventing a temporary authentication/authorization system while SEC-001/SEC-002 remain NOT_STARTED.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/catalog/{lib/mongo-errors.ts+test, models/brand.model.ts, repositories/brand.repository.ts+test, services/brand.service.ts+test, validation/brand.schema.ts} (8 new files); catalog README.md extended with a Brand section; category.repository.ts modified only to import the extracted shared helper (Category behavior and tests unchanged, verified). No new dependency; no route registered.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business CRUD exposed over HTTP yet, no auth/RBAC. The category.repository.ts change is a pure, behavior-preserving extraction, confirmed by all pre-existing CAT-001 tests remaining green.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved with one required adjustment (shared mongo-errors extraction) before execution</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>92af3b679a5bbfe2dbe08719d1161cfc755ebe12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record SEC-001 completion
Marks SEC-001 COMPLETED in MASTER_TASK_LIST.xlsx, adds the
DEVELOPMENT_PROGRESS.xlsx row and CHANGE_LOG.xlsx entry (CHG-006),
logs the DEVELOPMENT_LOG.md entry, and records ADR-013 through
ADR-015 (hybrid JWT+session architecture, atomic refresh rotation
with family-wide reuse revocation, progressive login delay).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -742,8 +742,60 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CHG-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SEC-001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Implemented the authentication foundation: hybrid short-lived JWT access token (jose, HS256) plus DB-backed opaque rotating refresh token (SecuritySession), atomic compare-and-swap refresh rotation with family-wide reuse-detection revocation, absolute + sliding session expiry, registration/login with no account-existence enumeration, progressive login-failure delay (not a hard lockout), session listing/revocation, authenticate and CSRF middleware, cookie-based transport.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Establish the authentication foundation per MASTER_TASK_LIST SEC-001, as the prerequisite for SEC-002 (RBAC/organizations) and every customer/business module that requires an authenticated actor - without building RBAC, MFA, password reset, email verification, GeoIP, Redis, or the SEC-003 audit framework prematurely.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/auth/ directory (18 files) plus apps/api/src/middleware/{authenticate.ts+test,csrf.ts+test} and apps/api/src/lib/cookies.ts+test (24 new files total); apps/api/src/config/env.ts, lib/http-errors.ts, types/express.d.ts, app.ts, routes/v1/index.ts, package.json, .env.example modified to wire in the new module; 3 new dependencies (jose, @node-rs/argon2, cookie); 4 pre-existing test files (env.test.ts, connection.test.ts, health.route.test.ts, ready.route.test.ts) updated only to supply the newly-required JWT_ACCESS_TOKEN_SECRET in their local test config. No apps/api/src/modules/catalog/ file touched.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Medium - this is the first module with real session/credential handling. Mitigated by: atomic (not read-then-write) refresh rotation proven by a dedicated concurrency test; family-wide revocation on reuse detection; generic, non-enumerating responses for every registration/login/refresh failure mode; progressive login delay instead of a lockout an attacker could weaponize against a victim; CSRF double-submit plus Origin/Referer validation; no plaintext secret ever logged (verified by a dedicated test). authenticate() intentionally performs no per-request DB lookup, a documented, accepted tradeoff for short-lived access tokens.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after a revision round covering atomic rotation, session-family design, absolute lifetime, CSRF scope, registration/lockout behavior, and cookie-parsing verification, before execution</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>aaffd29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record SEC-002 completion
Marks SEC-002 COMPLETED in MASTER_TASK_LIST.xlsx, adds the
DEVELOPMENT_PROGRESS.xlsx row and CHANGE_LOG.xlsx entry (CHG-007),
logs the DEVELOPMENT_LOG.md entry, and records ADR-016 through
ADR-018 (fixed role enum + static permissions, URL-based organization
context re-verified per request, atomic-counter last-owner
protection).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -794,8 +794,60 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CHG-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SEC-002</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Implemented the RBAC foundation: Organization and OrganizationMembership (User has no organizationId), fixed OWNER/ADMIN/MEMBER roles with a static role-to-permission map (no Role/Permission collections), URL-based organization context re-verified server-side on every request via resolveOrganizationContext(), and atomic activeOwnerCount-based last-owner protection. Organization creation and the first OWNER membership are one atomic withTransaction() unit.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Establish the authorization foundation per MASTER_TASK_LIST SEC-002, as the prerequisite for tenant-scoped access to catalog and every future business module - without building RBAC UI, dynamic/custom roles, platform-admin functionality, or the SEC-003 audit framework prematurely.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/organizations/ directory (21 files); apps/api/src/lib/http-errors.ts (+FORBIDDEN/ForbiddenError) and apps/api/src/routes/v1/index.ts (mount /organizations) modified to wire in the new module. No new dependencies. No apps/api/src/modules/auth/, modules/catalog/, db/, or SEC-001 middleware/types file touched.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Medium - this is the first module enforcing cross-user/cross-organization access control. Mitigated by: a dedicated concurrency test proving the true write-skew race (two different owners demoted/removed concurrently) is correctly rejected by the atomic counter, not just a same-document race; an atomic bootstrap transaction with a rollback test; byte-identical generic 403s across all three organization-context failure reasons (no enumeration); and mass-assignment-proof membership creation (strict schema plus a service signature with no role/status parameter at all). Suspension has an accepted, deliberate limitation: no role, including OWNER, can reactivate a SUSPENDED organization within SEC-002 - by explicit instruction, not an oversight.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after two revision rounds covering atomic bootstrap, last-owner concurrency strategy, the exact permission matrix, suspension semantics, membership lifecycle/indexing, mass-assignment protection, self-management edge cases, organization-context verification, and the req.membership/Express-declaration-merging approach, before execution</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>358b2e2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record SEC-003 completion
Marks SEC-003 COMPLETED in MASTER_TASK_LIST.xlsx, adds the
DEVELOPMENT_PROGRESS.xlsx row and CHANGE_LOG.xlsx entry (CHG-008),
logs the DEVELOPMENT_LOG.md entry, and records ADR-019 (single
append-only AuditEvent collection, post-commit writes, best-effort
semantics).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -846,8 +846,60 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CHG-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SEC-003</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Implemented the audit event infrastructure: a single append-only AuditEvent collection (no separate SecurityEvent), wired into the 13 sensitive actions verified reachable in the existing SEC-001 (auth) and SEC-002 (organizations) code. Audit writes for transactional operations happen strictly after commit, never inside a withTransaction() callback. Writes are best-effort and non-blocking. auth.login.failure never populates actorUserId/entityId. organization.reactivated is not instrumented since it cannot currently occur.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Establish the audit trail per MASTER_TASK_LIST SEC-003, satisfying "sensitive actions create safe audit events" for the security-domain actions that already exist, without inventing audit events for business modules (catalog, orders, payments) that have no route layer yet.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/audit/ directory (6 files); apps/api/src/modules/auth/services/auth.service.ts (+optional logger param on 5 functions, +13 audit calls) and routes/auth.route.ts (5 one-line edits); apps/api/src/modules/organizations/services/{organization,membership}.service.ts (+audit calls, no signature change). Additive-only test changes in 4 existing test files. No new dependencies. No modules/catalog, db/, middleware/authenticate.ts, middleware/csrf.ts, middleware/rate-limit.ts, or types/express.d.ts file touched.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Low-Medium - write-only infrastructure with no read/query surface yet, so no new attack surface for unauthorized data access. Mitigated by: audit writes placed after transaction commit (avoids duplicate records from MongoDB's transient-error retry), best-effort/non-blocking semantics (an audit outage cannot become a login/organization-mutation outage), three-layer metadata safety (scalar-only type, explicit per-call-site construction, forbidden-key runtime backstop) preventing secret leakage into audit records, and locked actor-omission semantics preventing a failed-login target from being misrepresented as a verified actor.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after two revision rounds covering transaction timing, failed-login auditing and its coexistence with LoginAttempt, the exact locked action matrix (including explicitly excluding the unreachable organization.reactivated), the auth.service.ts call-graph inspection confirming the minimal optional-parameter change, metadata-safety mechanism, and tenant-context sourcing, before execution</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>b10e976</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J8"/>
+  <autoFilter ref="A1:J9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record CAT-003 completion
Marks CAT-003 COMPLETED in MASTER_TASK_LIST.xlsx, adds the
DEVELOPMENT_PROGRESS.xlsx row and CHANGE_LOG.xlsx entry (CHG-009),
logs the DEVELOPMENT_LOG.md entry, and records ADR-020 (Product
references Category/Brand with organization-scoped, non-archived
validation and no cascade on later archiving).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -898,8 +898,60 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CHG-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CAT-003</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Implemented the Product domain foundation: Mongoose model, repository, and service (Service -&gt; Repository -&gt; Model, matching CAT-001/CAT-002 exactly), organization-scoped optional single categoryId and optional brandId references (both validated organization-scoped and non-archived, mirroring Category's own parent-validation pattern), optional media array (max 10 items), DRAFT/ACTIVE/ARCHIVED soft-archive lifecycle. No SKU, barcode, price, cost, inventory, or attributes - all explicitly Variant/CAT-004 responsibility.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Establish the Product foundation per MASTER_TASK_LIST CAT-003, reusing CAT-001/CAT-002 conventions (slugify, common validation helpers, lifecycle enum shape, cross-reference validation pattern) without prematurely building Variant (CAT-004), routes, or audit-event wiring.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/catalog/{models/product.model.ts, repositories/product.repository.ts+test, services/product.service.ts+test, validation/product.schema.ts} (6 new files); catalog README.md extended with a Product section. No existing CAT-001/CAT-002 file modified; no new dependency; no route registered; no audit event wired.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business logic exposed over HTTP yet, no auth/RBAC wiring, no audit integration. Category/Brand reference validation reuses an already-proven pattern (Category's own assertValidParent) rather than inventing a new one. Archiving a referenced Category/Brand never cascades onto an existing Product, verified by a dedicated test.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved with explicit locked decisions on categoryId/brandId optionality and cardinality, media shape/cap, archived-reference policy, and continued route/audit deferral, before execution</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0cb8ca2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record CAT-004 completion
Updates MASTER_TASK_LIST.xlsx (CAT-004 -> COMPLETED), DEVELOPMENT_PROGRESS.xlsx,
CHANGE_LOG.xlsx (CHG-010), DEVELOPMENT_LOG.md, and ARCHITECTURE_DECISIONS.md
(ADR-021) for the ProductVariant foundation implemented in b98a0ea.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -950,8 +950,60 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CHG-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CAT-004</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Implemented the ProductVariant domain foundation: Mongoose model, repository, and service (Service -&gt; Repository -&gt; Model, matching CAT-001/002/003), required immutable productId reference validated like Product's own Category/Brand pattern, organization-scoped unique SKU (uppercase-normalized), optional organization-scoped unique barcode (partial index), integer-minor-unit pricing (price required, compareAtPrice/cost optional, per existing ADR-008), and a prototype-pollution-safe {key,value}[] attribute array capped at 30 items. DRAFT/ACTIVE/ARCHIVED lifecycle, unrestricted transitions for consistency with Category/Brand/Product.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Establish the ProductVariant foundation per MASTER_TASK_LIST CAT-004, adding the SKU/pricing/attribute/lifecycle layer CAT-003 deliberately excluded from Product, without inventing inventory, currency, variant media, or routes/audit infrastructure not required by this task.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/catalog/{models/product-variant.model.ts, repositories/product-variant.repository.ts+test, services/product-variant.service.ts+test, validation/product-variant.schema.ts} (6 new files); catalog README.md extended with a ProductVariant section. No existing CAT-001/CAT-002/CAT-003 file modified; no new dependency; no route registered; no audit event wired.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Low - foundation-only, no business logic exposed over HTTP yet, no auth/RBAC wiring, no audit integration. Product reference validation reuses an already-proven pattern (Product's own assertValidCategory/assertValidBrand) rather than inventing a new one. A barcode sparse-index approach was tried first, found not to behave as intended on a compound index (organizationId is always present, so sparse never excluded a barcode-less document), and corrected to a partialFilterExpression index before this was committed - caught by a failing test, not left as a known defect.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved with 12 explicit locked decisions on SKU/barcode/money/attribute/lifecycle/relationship/inventory/media/display-name/routes/audit design, plus two modifications (no digits-only/checksum barcode validation, no compareAtPrice&gt;=price enforcement yet), before execution</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>b98a0ea</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
+  <autoFilter ref="A1:J11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record INV-001 completion
Updates MASTER_TASK_LIST.xlsx (INV-001 -> COMPLETED), DEVELOPMENT_PROGRESS.xlsx,
CHANGE_LOG.xlsx (CHG-011), DEVELOPMENT_LOG.md (also backfilling the CAT-004
security-review test commit 5805a17), and ARCHITECTURE_DECISIONS.md
(ADR-022) for the inventory engine implemented in 95105c6.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1002,8 +1002,60 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CHG-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Implemented the inventory engine: Location, StockBalance, and an append-only InventoryTransaction ledger. quantityOnHand is never directly patchable - only atomic incrementOrCreate/decrementIfSufficient operations exist, both requiring an active session. recordTransaction() handles PURCHASE/SALE/RETURN/ADJUSTMENT/DAMAGE/OPENING_BALANCE; a dedicated recordTransfer() atomically moves stock between two locations and writes matching TRANSFER_OUT/TRANSFER_IN entries, never via two independent recordTransaction() calls.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Establish the inventory foundation per MASTER_TASK_LIST INV-001, extending ADR-018's atomic-guarded-counter pattern to a new domain and reusing the append-only-collection pattern SEC-003 already established for AuditEvent, without prematurely building purchasing (BUS-001), POS (BUS-004), cart/checkout integration, pricing, currency, or SEC-003 audit wiring.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/inventory/ directory (18 files, all new). No existing CAT-001/002/003/004, auth, organizations, audit, db, or middleware file modified; no new dependency; no route registered; no audit event wired.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Medium - this is the first catalog-adjacent module requiring multi-document MongoDB transactions (ledger write + balance update must succeed or fail together) and the first requiring genuine concurrent-write correctness guarantees for a mutable aggregate. Mitigated by directly reusing ADR-018's already-proven atomic-guarded-decrement pattern rather than inventing a new one, and by two mandatory concurrency tests (concurrent initial-balance creation with no lost update, concurrent outbound operations with no negative balance) both passing against a real MongoDB replica set. A real defense-in-depth gap (a Mongoose custom validator silently not firing for an undefined ADJUSTMENT direction) was found and fixed during testing, not left as a known issue.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after two revision rounds covering the Location/StockBalance/InventoryTransaction split, ADJUSTMENT direction semantics, the dedicated recordTransfer() operation, the atomic guarded-decrement requirement, mandatory concurrency test scenarios with exact numeric expectations, and explicit exclusion of audit wiring, forward-looking foreign keys, currency, and negative-inventory configuration, before execution</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>95105c6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J11"/>
+  <autoFilter ref="A1:J12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record CUST-001 completion
Updates MASTER_TASK_LIST.xlsx (CUST-001 -> COMPLETED), DEVELOPMENT_PROGRESS.xlsx,
CHANGE_LOG.xlsx (CHG-012), DEVELOPMENT_LOG.md (also backfilling the INV-001
security-review test commit 5747c1e), ARCHITECTURE_DECISIONS.md (ADR-023),
and OPEN_DECISIONS.md (DEC-007: the SEC-003 audit-wiring conflict for
customer.archived/customer.restored, left unresolved for a follow-up
decision) for the customer accounts module implemented in c3ab6a5.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1054,8 +1054,60 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CHG-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Implemented Customer accounts: a global (non-organization-scoped) Customer profile 1:1 with User, and a separate Address collection supporting multiple addresses per customer with database-enforced at-most-one default billing/one default shipping via partial unique indexes. Added the first HTTP route layer outside SEC-001/SEC-002 (self-service /api/v1/customers/me... endpoints, identity always from req.auth.userId). setDefaultAddress runs inside one withTransaction().</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Establish the customer-account foundation per MASTER_TASK_LIST CUST-001, deliberately keeping Customer global (not organization-scoped) to match User's own precedent and the future marketplace direction, and adding routes now because the acceptance criterion ("Customer account flows work securely") is inherently a self-service HTTP flow, unlike the catalog/inventory foundation tasks.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/customers/ directory (17 new files); apps/api/src/routes/v1/index.ts modified only to mount the new router (2 hunks: import + router.use). No CAT-001-004, INV-001, auth, organizations, audit, or db file modified; no new dependency.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Medium - the first module to add a route layer since SEC-002, and the first to use a MongoDB transaction for a non-inventory purpose (default-address switching). Mitigated by: every route resolving identity exclusively from req.auth.userId (never a client-supplied id); every address repository function requiring customerId as a mandatory scoping parameter; a dedicated concurrency test proving two simultaneous setDefaultAddress calls resolve to exactly one default; a transaction-rollback test proving an archived-target default-swap attempt leaves the prior default untouched. One approved decision could not be fully implemented as specified: customer.archived/customer.restored audit events were approved but conflict with the explicit "do not modify SEC-003" boundary (wiring them requires extending SEC-003's own AUDIT_ACTIONS enum) - resolved by not touching SEC-003 and flagging the conflict explicitly (module README + a test proving the current zero-audit-event state) rather than silently choosing a side.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after one revision round covering organization scope (global, not org-scoped), routes (approved now, self-service only), customer status (dedicated archive/restore only), address lifecycle (soft delete), the default-address transaction requirement (changed from two independent writes to one withTransaction() per explicit instruction), audit scope (customer.archived/restored only), and the country field (bounded free-text, no dependency), before execution</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>c3ab6a5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): resolve DEC-007 (customer audit wiring)
Moves DEC-007 to a resolved-decisions table in OPEN_DECISIONS.md,
records the resolution as an addendum to ADR-023 (no new ADR - a
clarification of the existing decision, not a new one), adds CHG-013
to CHANGE_LOG.xlsx, and appends a DEVELOPMENT_LOG.md entry for the
customer.archived/customer.restored audit wiring implemented in
a7656f9.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1106,8 +1106,60 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CHG-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Customer / Audit</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Resolved DEC-007: extended SEC-003's AUDIT_ACTIONS/AUDIT_ENTITY_TYPES with customer.archived, customer.restored, and Customer (an 8-line additive change to modules/audit/models/audit-event.model.ts, no existing action/entity/behavior touched). Wired archiveCustomerProfile()/restoreCustomerProfile() to call the existing audit.service.ts record() after a successful archive/restore, with actorUserId from the authenticated userId and entityId the Customer._id.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CUST-001's approved audit requirement (customer.archived/customer.restored) directly conflicted with that same task's "do not modify SEC-003" boundary. The conflict was recorded (DEC-007) rather than resolved unilaterally; the developer subsequently approved the small additive SEC-003 extension as the resolution.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Modified apps/api/src/modules/audit/models/audit-event.model.ts (+8 lines: two new AUDIT_ACTIONS entries, one new AUDIT_ENTITY_TYPES entry, one explanatory comment). Modified apps/api/src/modules/customers/services/customer.service.ts (audit wiring in archiveCustomerProfile/restoreCustomerProfile, optional trailing logger parameter added to both) and apps/api/src/modules/customers/routes/customer.route.ts (logger passthrough on DELETE /me). No other SEC-003 file modified (repository, service internals, error handling, metadata rules all unchanged). No CAT-001-004, INV-001, auth, or organizations file touched.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Low - purely additive to a locked enum, with the existing best-effort/non-blocking audit.service.ts record() reused unchanged. Mitigated by: 5 new/rewritten tests proving exactly one customer.archived/customer.restored event per successful operation with the correct actorUserId/entityType/entityId, zero events for ordinary profile/address CRUD, and zero events for a failed (NotFoundError) archive/restore attempt; SEC-003's own 12 existing tests re-run in isolation and confirmed unaffected; full regression (CAT-001-004, INV-001, auth, organizations) re-verified unchanged.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - explicit approval of the small additive SEC-003 extension as the resolution to DEC-007, with 13 numbered requirements (exact actions to add, no SEC-003 redesign, actor/entity source, no new audit API, no CRUD/address-lifecycle auditing) specified before execution</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>a7656f9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J13"/>
+  <autoFilter ref="A1:J14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record COM-001 completion
Updates MASTER_TASK_LIST.xlsx (COM-001 -> COMPLETED), DEVELOPMENT_PROGRESS.xlsx,
CHANGE_LOG.xlsx (CHG-014), DEVELOPMENT_LOG.md, and ARCHITECTURE_DECISIONS.md
(ADR-024) for the wishlist and back-in-stock request module implemented
in 183c87d.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1158,8 +1158,60 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CHG-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>COM-001</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Implemented Wishlist and BackInStockRequest: two separate collections referencing a global Customer and an organization-owned ProductVariant. Partial unique indexes ({customerId,variantId} scoped to status:ACTIVE, {customerId,variantId,status} scoped to status:PENDING) permit re-adding/re-requesting after soft-removal/cancellation while preventing duplicates while active. Back-in-stock requests require aggregate stock (all locations) to be zero, checked via INV-001's existing repository, unmodified. Added the second self-service HTTP route layer (after CUST-001).</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Establish the wishlist/back-in-stock foundation per MASTER_TASK_LIST COM-001, deliberately stopping at "saved and requested" per the task's own acceptance wording - no notification delivery (DEC-003/DEC-004 unresolved, no queue infrastructure) and no FULFILLED/fulfillment-detection logic (would require modifying INV-001 or inventing job infrastructure).</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/wishlist/ directory (18 new files); apps/api/src/routes/v1/index.ts modified only to mount the new router. No CAT-001-004, INV-001, CUST-001, auth, organizations, audit, or db file modified; no new dependency.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Medium - the first module to validate an organization reference without using SEC-002's membership middleware (a new, deliberately narrower read-only existence+ACTIVE check was needed, since customers are not organization members), and the first to layer a cross-collection stock aggregation read (INV-001) underneath a create-time validation rule. Mitigated by: the authoritative tenant check remaining ProductVariant's own organization-scoped lookup, never the client-supplied organizationId alone; concurrent-create race tests for both partial unique indexes; all four required multi-location stock scenarios tested explicitly. One real regression was found and fixed during validation, not left as a known issue: the wishlist router's initially-blanket authenticate() middleware incorrectly 401'd genuinely unmatched, unrelated routes (caught by the pre-existing health.route.test.ts regression test), corrected by scoping the middleware to the router's own two path prefixes before this task was considered complete.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after one revision round, then implementation approved with 24 numbered requirements covering organization-scoping validation flow, customer-identity resolution, both partial-unique-index designs with mandatory re-add/re-request and concurrency tests, multi-location stock semantics with four explicit test scenarios, archived-variant/archived-customer write-blocking, route shape and request bodies, cross-module reuse boundaries, and explicit exclusion of FULFILLED/notification-delivery/SEC-003 audit wiring, before execution</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>183c87d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J14"/>
+  <autoFilter ref="A1:J15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record COM-002 completion
Marks COM-002 COMPLETED in MASTER_TASK_LIST.xlsx, records the
implementation in DEVELOPMENT_PROGRESS.xlsx and DEVELOPMENT_LOG.md,
logs CHG-015 in CHANGE_LOG.xlsx, and records ADR-025 (Cart: one Cart
per customer per organization, dynamic pricing and server-computed
totals) in ARCHITECTURE_DECISIONS.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1210,8 +1210,60 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CHG-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>COM-002</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Implemented Cart and CartItem: one Cart per (customerId, organizationId), CartItem as a separate, hard-deleted collection carrying only {cartId, organizationId, variantId, quantity} - no price/name/SKU snapshot. Every price/subtotal/total in GET /cart is resolved live from the current ProductVariant/Product on every call. The 1..9999 per-item quantity ceiling is enforced entirely inside a single atomic MongoDB operation (filter-embedded ceiling check + $inc + upsert), never a read-calculate-write sequence. GET and the clear-cart operation never create a Cart; only POST /cart/items does (via an atomic findOrCreate).</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Establish the Cart foundation per MASTER_TASK_LIST COM-002 ("Cart lifecycle and server-side pricing validation," acceptance: "Cart totals are server-authoritative"), reusing COM-001's read-only organization/variant validation pattern and INV-001's unmodified stock-balance read for an informational availability indicator, without inventing inventory reservation, discount/tax/shipping calculation, or a Cart lifecycle/status field beyond what this task requires.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/cart/ directory (14 new files); apps/api/src/routes/v1/index.ts modified only to mount the new router under a '/cart' prefix. No CAT-001-004, INV-001, CUST-001, COM-001, auth, organizations, audit, or db file modified; no new dependency.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Medium - the first module in this codebase to enforce a numeric ceiling atomically inside a single upsert-increment MongoDB operation rather than a separate read-then-write step (mitigated by two dedicated concurrency race tests: 5000+5000 exceeding 9999 resolves to exactly one success, 3000+3000 staying within it applies both), and the first CartItem-style collection to use a hard delete plus a plain (non-partial) unique index instead of this codebase's usual soft-delete-with-partial-index pattern (a deliberate, reasoned deviation, not an oversight, since a cart item has no history value once removed). CartItem carries no customerId (unlike WishlistItem/BackInStockRequest), so item-level ownership is resolved via a two-step cartId-then-Cart.customerId check rather than a single-collection scoped query - proven safe by dedicated cross-customer IDOR tests at the service and route layers.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after a detailed 30-section repository audit, then implementation approved with explicit mandatory corrections: the 9999 ceiling enforced atomically (with 9990+9/9990+20 required test scenarios), GET must never create a Cart, and archived-variant handling specified per-operation (POST/PATCH reject, DELETE always allowed, GET shows flagged) - before execution</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>5a0639f</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J15"/>
+  <autoFilter ref="A1:J16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): record COM-003 completion
Marks COM-003 COMPLETED in MASTER_TASK_LIST.xlsx, records the
implementation in DEVELOPMENT_PROGRESS.xlsx and DEVELOPMENT_LOG.md,
logs CHG-016 in CHANGE_LOG.xlsx, and records ADR-026 (Checkout:
preview/confirm, server revalidation, order creation and atomic cart
clearing) in ARCHITECTURE_DECISIONS.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1262,8 +1262,60 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CHG-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>COM-003</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Implemented Checkout preview/confirm and a new minimal orders module: Order {customerId, organizationId, items[] embedded snapshot, subtotal, total, status: PENDING_PAYMENT, shippingAddress/billingAddress embedded snapshot}. Preview and confirm share one pricing/validation function that always re-resolves current ProductVariant.price/Product.name and validates aggregate StockBalance (read-only, INV-001 unmodified). Order creation and Cart clearing happen inside one withTransaction(), re-reading Cart/CartItem via the transaction's own session by importing COM-002's public Cart/CartItem models directly (their repositories do not accept a session, and COM-002 is closed).</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Establish the Checkout foundation per MASTER_TASK_LIST COM-003 ("Checkout preview and order creation," acceptance: "Checkout validates stock, price and customer data"), taking the roadmap's own wording literally so COM-003, not COM-004, creates the first Order - COM-004 ("Order lifecycle, tracking, cancellation and returns") is scoped to managing an already-existing order's state machine, not creating one.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/checkout/ (9 files) and apps/api/src/modules/orders/ (5 files), all new; apps/api/src/routes/v1/index.ts modified only to mount the new router under /checkout. No CAT-001-004, INV-001, CUST-001, COM-001, COM-002, auth, organizations, audit, or db file modified; no new dependency.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Medium-high - the first module to open a MongoDB transaction whose read step (re-reading Cart/CartItem via the session) reaches into another, already-closed module's Mongoose models directly rather than through that module's own repository layer, specifically because COM-002's repositories do not accept a ClientSession and modifying a closed module was out of scope. Mitigated by: read+delete only (never a write of new Cart data), documented explicitly in both modules' READMEs, and proven safe by a genuine concurrent-confirm race test (two simultaneous confirms for the same cart resolve to exactly one Order, the loser correctly seeing an empty cart via MongoDB's own write-conflict-plus-retry behavior - no bespoke idempotency-key infrastructure needed for that specific race). A second, separate, explicitly-flagged risk: a client retry after a lost HTTP response following a successful commit will see an empty cart rather than being replayed the original order - a known, deliberately deferred limitation, not a silently accepted one.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - plan approved after a detailed 35-section repository audit that surfaced and required an explicit ruling on a tension in the roadmap's own wording (whether COM-003 or COM-004 creates the initial Order), then implementation approved with 3 core invariants stated as non-negotiable (server-authoritative price/totals, inventory validation without mutation, atomic Order-creation-plus-Cart-clearing) plus detailed, mandatory address/pricing/transaction/concurrency requirements, before execution</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>9bd3bfe</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J16"/>
+  <autoFilter ref="A1:J17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planning): close COM-004 F-1 remediation
Records COM-004 Tranche A (order lifecycle state machine, customer
cancel/tracking, return-request creation/listing, ReturnRequestLock
concurrency mechanism — commit 5af12bd) and the F-1 security-review
remediation (duplicate-variantId quantity-invariant bypass, fixed in
commit 43d1af1 and independently re-verified PASS) in
MASTER_TASK_LIST.xlsx, DEVELOPMENT_PROGRESS.xlsx, CHANGE_LOG.xlsx
(CHG-017), and DEVELOPMENT_LOG.md.

COM-004 is set to IN_PROGRESS rather than COMPLETED: Tranche B
(staff/admin order management, payment/refund integration, inventory
decrement, return-window enforcement, return approve/reject/receive)
remains open within the same task row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning/CHANGE_LOG.xlsx
+++ b/Planning/CHANGE_LOG.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1314,8 +1314,60 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CHG-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>COM-004</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Implemented COM-004 Tranche A: Order lifecycle state machine (PENDING_PAYMENT -&gt; CONFIRMED -&gt; PROCESSING -&gt; PACKED -&gt; SHIPPED -&gt; DELIVERED, plus CANCELLED from PENDING_PAYMENT/CONFIRMED only), every transition enforced by an atomically-guarded findOneAndUpdate (filter embeds the required fromStatus, never read-then-write); customer order list/detail/cancel APIs; tracking fields (carrier, trackingNumber, shippedAt, deliveredAt); a new returns module (ReturnRequest, customer-only create/list, backed by a dedicated ReturnRequestLock collection that serializes concurrent submissions against the same order via MongoDB write-conflict detection plus automatic transaction retry). SEC-003's AuditEvent additively extended with order.status_changed, order.cancelled, return.requested. During the mandatory post-implementation security review, finding F-1 (HIGH) was identified: a single return-request payload repeating the same variantId bypassed the purchased-quantity/cumulative-quantity invariant, since both the Order-snapshot check and the in-transaction cumulative check validated each item entry independently instead of by aggregate. Remediated with schema-level duplicate-variantId rejection plus independent service-layer per-variant quantity aggregation (defense-in-depth, not reliance on schema validation alone), 4 new regression tests, and a subsequent independent follow-up security review that returned PASS with no new findings.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Establish the Order lifecycle required by COM-004's own MASTER_TASK_LIST acceptance criterion ("State transitions are controlled and tested"), with returns modeled as a separate ReturnRequest collection rather than an Order.status value, per the approved plan. F-1 was remediated because a financial/inventory-integrity invariant must not rely solely on schema validation, per explicit developer requirement.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>New apps/api/src/modules/returns/ module (models, repositories, service, validation, README); apps/api/src/modules/orders/ extended (model, repository, service, validation, route, README); apps/api/src/modules/audit/models/audit-event.model.ts additively extended (3 new AUDIT_ACTIONS, 2 new AUDIT_ENTITY_TYPES); apps/api/src/routes/v1/index.ts modified only to mount the orders router. No CAT-001-004, INV-001, CUST-001, COM-001, COM-002, COM-003 checkout files, auth, organizations, or db file modified; no new dependency. 139 new tests across the implementation and the F-1 remediation (891/891 total passing, zero regression).</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Medium - the first insert-based (not update/delete-based) multi-document invariant in this codebase: MongoDB transaction isolation does not naturally serialize two concurrent transactions that each insert a different new document, so ReturnRequestLock (one document per orderId, atomically upserted inside the transaction before the aggregate read) was introduced to force write-conflict detection and automatic retry - proven by dedicated concurrency tests. The HIGH-severity F-1 finding was caught by the mandatory security review before this Planning entry was ever recorded, fixed, and independently re-verified PASS - consistent with the explicit instruction that Planning/completion records be held back until the security-review workflow passes. Tranche B (staff/admin order management, payment/refund integration, inventory decrement, return-window enforcement, return approve/reject/receive) remains open; COM-004 is recorded as IN_PROGRESS, not COMPLETED, in MASTER_TASK_LIST.xlsx.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Developer (via this conversation) - Tranche A scope, the ReturnRequestLock concurrency design, and explicit SEC-003 action names approved before implementation; the F-1 remediation scope and required defense-in-depth approach approved separately after the initial security review returned BLOCKED; this closure recorded after an independent follow-up security review returned PASS</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>5af12bd (Tranche A implementation), 43d1af1 (F-1 remediation)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J17"/>
+  <autoFilter ref="A1:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>